<commit_message>
updated by 28April2025 from CRMAC Desktop
</commit_message>
<xml_diff>
--- a/BOND_EQT/RAI.xlsx
+++ b/BOND_EQT/RAI.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c060ac0a7f9c7ae2/main/DELL_NB/EU/BOND_EQT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="11_F25DC773A252ABDACC1048DAA15A48A85ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0B7BBED-9DCA-4A8B-A6CE-5BC9F675D647}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_F25DC773A252ABDACC1048DAA15A48A85ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BABE24B-632B-4258-9459-30ADE72209AB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="480" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -365,7 +365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3961"/>
+  <dimension ref="A1:E3995"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -43944,6 +43944,380 @@
         <v>-0.12189999999999999</v>
       </c>
     </row>
+    <row r="3962" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3962" s="1">
+        <v>45723</v>
+      </c>
+      <c r="B3962" s="2">
+        <v>-0.2392</v>
+      </c>
+      <c r="C3962" s="2">
+        <v>0.2104</v>
+      </c>
+    </row>
+    <row r="3963" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3963" s="1">
+        <v>45726</v>
+      </c>
+      <c r="B3963" s="2">
+        <v>-0.4093</v>
+      </c>
+      <c r="C3963" s="2">
+        <v>-3.1399999999999997E-2</v>
+      </c>
+    </row>
+    <row r="3964" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3964" s="1">
+        <v>45727</v>
+      </c>
+      <c r="B3964" s="2">
+        <v>-0.33839999999999998</v>
+      </c>
+      <c r="C3964" s="2">
+        <v>0.1134</v>
+      </c>
+    </row>
+    <row r="3965" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3965" s="1">
+        <v>45728</v>
+      </c>
+      <c r="B3965" s="2">
+        <v>-0.24360000000000001</v>
+      </c>
+      <c r="C3965" s="2">
+        <v>0.2621</v>
+      </c>
+    </row>
+    <row r="3966" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3966" s="1">
+        <v>45729</v>
+      </c>
+      <c r="B3966" s="2">
+        <v>-0.4199</v>
+      </c>
+      <c r="C3966" s="2">
+        <v>5.2699999999999997E-2</v>
+      </c>
+    </row>
+    <row r="3967" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3967" s="1">
+        <v>45730</v>
+      </c>
+      <c r="B3967" s="2">
+        <v>-0.26910000000000001</v>
+      </c>
+      <c r="C3967" s="2">
+        <v>0.2462</v>
+      </c>
+    </row>
+    <row r="3968" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3968" s="1">
+        <v>45733</v>
+      </c>
+      <c r="B3968" s="2">
+        <v>-0.191</v>
+      </c>
+      <c r="C3968" s="2">
+        <v>0.23180000000000001</v>
+      </c>
+    </row>
+    <row r="3969" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3969" s="1">
+        <v>45734</v>
+      </c>
+      <c r="B3969" s="2">
+        <v>-0.12509999999999999</v>
+      </c>
+      <c r="C3969" s="2">
+        <v>0.22120000000000001</v>
+      </c>
+    </row>
+    <row r="3970" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3970" s="1">
+        <v>45735</v>
+      </c>
+      <c r="B3970" s="2">
+        <v>-0.1057</v>
+      </c>
+      <c r="C3970" s="2">
+        <v>0.26600000000000001</v>
+      </c>
+    </row>
+    <row r="3971" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3971" s="1">
+        <v>45736</v>
+      </c>
+      <c r="B3971" s="2">
+        <v>-0.14729999999999999</v>
+      </c>
+      <c r="C3971" s="2">
+        <v>0.27060000000000001</v>
+      </c>
+    </row>
+    <row r="3972" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3972" s="1">
+        <v>45737</v>
+      </c>
+      <c r="B3972" s="2">
+        <v>-0.20369999999999999</v>
+      </c>
+      <c r="C3972" s="2">
+        <v>0.2387</v>
+      </c>
+    </row>
+    <row r="3973" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3973" s="1">
+        <v>45740</v>
+      </c>
+      <c r="B3973" s="2">
+        <v>-7.5899999999999995E-2</v>
+      </c>
+      <c r="C3973" s="2">
+        <v>0.38769999999999999</v>
+      </c>
+    </row>
+    <row r="3974" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3974" s="1">
+        <v>45741</v>
+      </c>
+      <c r="B3974" s="2">
+        <v>-7.9699999999999993E-2</v>
+      </c>
+      <c r="C3974" s="2">
+        <v>0.37240000000000001</v>
+      </c>
+    </row>
+    <row r="3975" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3975" s="1">
+        <v>45742</v>
+      </c>
+      <c r="B3975" s="2">
+        <v>-0.1676</v>
+      </c>
+      <c r="C3975" s="2">
+        <v>0.28289999999999998</v>
+      </c>
+    </row>
+    <row r="3976" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3976" s="1">
+        <v>45743</v>
+      </c>
+      <c r="B3976" s="2">
+        <v>-0.31140000000000001</v>
+      </c>
+      <c r="C3976" s="2">
+        <v>0.2185</v>
+      </c>
+    </row>
+    <row r="3977" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3977" s="1">
+        <v>45744</v>
+      </c>
+      <c r="B3977" s="2">
+        <v>-0.46329999999999999</v>
+      </c>
+      <c r="C3977" s="2">
+        <v>-8.0299999999999996E-2</v>
+      </c>
+    </row>
+    <row r="3978" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3978" s="1">
+        <v>45747</v>
+      </c>
+      <c r="B3978" s="2">
+        <v>-0.62480000000000002</v>
+      </c>
+      <c r="C3978" s="2">
+        <v>-0.29759999999999998</v>
+      </c>
+    </row>
+    <row r="3979" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3979" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B3979" s="2">
+        <v>-0.60629999999999995</v>
+      </c>
+      <c r="C3979" s="2">
+        <v>-0.27200000000000002</v>
+      </c>
+    </row>
+    <row r="3980" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3980" s="1">
+        <v>45749</v>
+      </c>
+      <c r="B3980" s="2">
+        <v>-0.5454</v>
+      </c>
+      <c r="C3980" s="2">
+        <v>-0.17849999999999999</v>
+      </c>
+    </row>
+    <row r="3981" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3981" s="1">
+        <v>45750</v>
+      </c>
+      <c r="B3981" s="2">
+        <v>-1.1372</v>
+      </c>
+      <c r="C3981" s="2">
+        <v>-0.82889999999999997</v>
+      </c>
+    </row>
+    <row r="3982" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3982" s="1">
+        <v>45751</v>
+      </c>
+      <c r="B3982" s="2">
+        <v>-1.6855</v>
+      </c>
+      <c r="C3982" s="2">
+        <v>-1.3678999999999999</v>
+      </c>
+    </row>
+    <row r="3983" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3983" s="1">
+        <v>45754</v>
+      </c>
+      <c r="B3983" s="2">
+        <v>-1.9251</v>
+      </c>
+      <c r="C3983" s="2">
+        <v>-1.6403000000000001</v>
+      </c>
+    </row>
+    <row r="3984" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3984" s="1">
+        <v>45755</v>
+      </c>
+      <c r="B3984" s="2">
+        <v>-1.7222999999999999</v>
+      </c>
+      <c r="C3984" s="2">
+        <v>-1.4858</v>
+      </c>
+    </row>
+    <row r="3985" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3985" s="1">
+        <v>45756</v>
+      </c>
+      <c r="B3985" s="2">
+        <v>-1.6588000000000001</v>
+      </c>
+      <c r="C3985" s="2">
+        <v>-1.3829</v>
+      </c>
+    </row>
+    <row r="3986" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3986" s="1">
+        <v>45757</v>
+      </c>
+      <c r="B3986" s="2">
+        <v>-1.3923000000000001</v>
+      </c>
+      <c r="C3986" s="2">
+        <v>-1.1536</v>
+      </c>
+    </row>
+    <row r="3987" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3987" s="1">
+        <v>45758</v>
+      </c>
+      <c r="B3987" s="2">
+        <v>-1.3179000000000001</v>
+      </c>
+      <c r="C3987" s="2">
+        <v>-1.1531</v>
+      </c>
+    </row>
+    <row r="3988" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3988" s="1">
+        <v>45761</v>
+      </c>
+      <c r="B3988" s="2">
+        <v>-1.1713</v>
+      </c>
+      <c r="C3988" s="2">
+        <v>-0.89129999999999998</v>
+      </c>
+    </row>
+    <row r="3989" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3989" s="1">
+        <v>45762</v>
+      </c>
+      <c r="B3989" s="2">
+        <v>-1.0914999999999999</v>
+      </c>
+      <c r="C3989" s="2">
+        <v>-0.74229999999999996</v>
+      </c>
+    </row>
+    <row r="3990" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3990" s="1">
+        <v>45763</v>
+      </c>
+      <c r="B3990" s="2">
+        <v>-1.1357999999999999</v>
+      </c>
+      <c r="C3990" s="2">
+        <v>-0.85509999999999997</v>
+      </c>
+    </row>
+    <row r="3991" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3991" s="1">
+        <v>45764</v>
+      </c>
+      <c r="B3991" s="2">
+        <v>-1.0448999999999999</v>
+      </c>
+      <c r="C3991" s="2">
+        <v>-0.68569999999999998</v>
+      </c>
+    </row>
+    <row r="3992" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3992" s="1">
+        <v>45765</v>
+      </c>
+      <c r="B3992" s="2">
+        <v>-1.0615000000000001</v>
+      </c>
+      <c r="C3992" s="2">
+        <v>-0.68</v>
+      </c>
+    </row>
+    <row r="3993" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3993" s="1">
+        <v>45768</v>
+      </c>
+      <c r="B3993" s="2">
+        <v>-1.0498000000000001</v>
+      </c>
+      <c r="C3993" s="2">
+        <v>-0.67059999999999997</v>
+      </c>
+    </row>
+    <row r="3994" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3994" s="1">
+        <v>45769</v>
+      </c>
+      <c r="B3994" s="2">
+        <v>-1.0125999999999999</v>
+      </c>
+      <c r="C3994" s="2">
+        <v>-0.57650000000000001</v>
+      </c>
+    </row>
+    <row r="3995" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3995" s="1">
+        <v>45770</v>
+      </c>
+      <c r="B3995" s="2">
+        <v>-0.79749999999999999</v>
+      </c>
+      <c r="C3995" s="2">
+        <v>-0.28949999999999998</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>